<commit_message>
chore: add product carousel captions
</commit_message>
<xml_diff>
--- a/content/social/content-calendar.xlsx
+++ b/content/social/content-calendar.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Calendar" sheetId="1" r:id="R9639479bd85248a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Calendar" sheetId="1" r:id="R5418a868524a44cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -936,10 +936,10 @@
 Visit the link in bio.</x:v>
       </x:c>
       <x:c r="J12" t="str">
-        <x:v>A full month of math practice, with reading passages, three levels, and answer keys in one packet.</x:v>
+        <x:v>Some months, the hardest part is keeping practice consistent. This November packet brings reading passages, three levels of math practice, and answer keys into one ready-to-use resource. Save this post, preview the pages, and find the full packet through the link in bio.</x:v>
       </x:c>
       <x:c r="K12" t="str">
-        <x:v>#teacherspayteachers #mathathome #homeschooling #printables</x:v>
+        <x:v>#novembermath #mathpractice #homeschoolmath #mathathome #teacherspayteachers #printableworksheets #elementarymath #homeschoolresources #mathresources #learningathome #printablelearning</x:v>
       </x:c>
       <x:c r="L12" t="str">
         <x:v>Planned</x:v>
@@ -987,10 +987,10 @@
 Get the full packet before the month begins.</x:v>
       </x:c>
       <x:c r="J13" t="str">
-        <x:v>November math practice is ready. Find the full packet through the link in bio.</x:v>
+        <x:v>November practice is ready. This packet brings reading passages, three levels of daily math practice, and answer keys into one place, so you can start the month with a plan. Preview the pages, then get the full packet through the link in bio.</x:v>
       </x:c>
       <x:c r="K13" t="str">
-        <x:v>#teacherspayteachers #mathathome #homeschooling #printables</x:v>
+        <x:v>#novembermath #mathpractice #homeschoolmath #mathathome #teacherspayteachers #printableworksheets #elementarymath #homeschoolresources #mathresources #learningathome #printablelearning</x:v>
       </x:c>
       <x:c r="L13" t="str">
         <x:v>Planned</x:v>

</xml_diff>